<commit_message>
Corrige #SPILL! na aba Séries: BDH em célula única (array dinâmico)
Substitui os arrays legados (CSE) de tamanho fixo por fórmulas BDH de
célula única, que derramam dinamicamente. Elimina o erro #SPILL! no
Excel moderno. Adiciona nota de troubleshooting nas instruções.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UySu8n7PttVLVLfLkuayDx
</commit_message>
<xml_diff>
--- a/pesquisa_xp_excel/MSCI_Brazil_EPS_Revisao_BBG.xlsx
+++ b/pesquisa_xp_excel/MSCI_Brazil_EPS_Revisao_BBG.xlsx
@@ -617,7 +617,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B34"/>
+  <dimension ref="B2:B36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -824,6 +824,20 @@
       <c r="B34" t="inlineStr">
         <is>
           <t>• Erros #N/A N/A: ticker inválido, sem histórico de estimativa, ou período fiscal indisponível para o índice.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>• #SPILL! na aba 'Séries': cada BDH é array dinâmico e precisa das linhas/colunas abaixo e à direita da célula</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  âncora (linha 4 de cada bloco) VAZIAS para derramar. Não cole nada nessa área; blocos já vêm espaçados.</t>
         </is>
       </c>
     </row>
@@ -1593,51 +1607,51 @@
     </row>
     <row r="4">
       <c r="A4">
-        <f t="array" ref="A4:B3003">BDH(Painel!$C$14,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$14,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="D4">
-        <f t="array" ref="D4:E3003">BDH(Painel!$C$15,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$15,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="G4">
-        <f t="array" ref="G4:H3003">BDH(Painel!$C$16,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$16,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="J4">
-        <f t="array" ref="J4:K3003">BDH(Painel!$C$17,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$17,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="M4">
-        <f t="array" ref="M4:N3003">BDH(Painel!$C$18,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$18,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="P4">
-        <f t="array" ref="P4:Q3003">BDH(Painel!$C$19,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$19,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="S4">
-        <f t="array" ref="S4:T3003">BDH(Painel!$C$20,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$20,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="V4">
-        <f t="array" ref="V4:W3003">BDH(Painel!$C$21,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$21,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="Y4">
-        <f t="array" ref="Y4:Z3003">BDH(Painel!$C$22,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$22,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="AB4">
-        <f t="array" ref="AB4:AC3003">BDH(Painel!$C$23,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$23,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="AE4">
-        <f t="array" ref="AE4:AF3003">BDH(Painel!$C$24,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$24,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
       <c r="AH4">
-        <f t="array" ref="AH4:AI3003">BDH(Painel!$C$25,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
+        <f>BDH(Painel!$C$25,"BEST_EPS",StartDate,EndDate,optPer,optFPer,optCcy,"Fill=P")</f>
         <v/>
       </c>
     </row>

</xml_diff>